<commit_message>
March 5 2024 v1
</commit_message>
<xml_diff>
--- a/_downloads/1ab64b1afe5c49044cdabd367bf46521/Ejercicios swap.xlsx
+++ b/_downloads/1ab64b1afe5c49044cdabd367bf46521/Ejercicios swap.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Swap\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DRIVE\Página cursos\source\Derivados financieros\Swap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D293083-44FE-4ADD-97C3-325BE349DDFB}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63BDD1C7-CE93-4915-A490-70C9ADDDC5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E59240A5-3B44-45EE-831B-FD90529A5C22}"/>
   </bookViews>
@@ -777,7 +777,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -801,7 +801,6 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -828,34 +827,26 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -873,15 +864,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -894,12 +876,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -910,15 +886,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -937,13 +907,13 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -973,7 +943,7 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -982,7 +952,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -997,10 +967,10 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1050,67 +1020,58 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4762,8 +4723,8 @@
       <xdr:row>31</xdr:row>
       <xdr:rowOff>6259</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 16">
@@ -5035,7 +4996,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 16">
@@ -5886,9 +5847,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5926,7 +5887,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -6032,7 +5993,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -6174,7 +6135,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -6194,126 +6155,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114"/>
-      <c r="I1" s="114"/>
-      <c r="J1" s="114"/>
-      <c r="K1" s="115"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="100"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B2" s="116"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="117"/>
-      <c r="H2" s="117"/>
-      <c r="I2" s="117"/>
-      <c r="J2" s="117"/>
-      <c r="K2" s="118"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="103"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="117"/>
-      <c r="H3" s="117"/>
-      <c r="I3" s="117"/>
-      <c r="J3" s="117"/>
-      <c r="K3" s="118"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102"/>
+      <c r="K3" s="103"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="118"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="103"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="117"/>
-      <c r="H5" s="117"/>
-      <c r="I5" s="117"/>
-      <c r="J5" s="117"/>
-      <c r="K5" s="118"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="103"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B6" s="116"/>
-      <c r="C6" s="117"/>
-      <c r="D6" s="117"/>
-      <c r="E6" s="117"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="117"/>
-      <c r="H6" s="117"/>
-      <c r="I6" s="117"/>
-      <c r="J6" s="117"/>
-      <c r="K6" s="118"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="102"/>
+      <c r="J6" s="102"/>
+      <c r="K6" s="103"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B7" s="116"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="117"/>
-      <c r="H7" s="117"/>
-      <c r="I7" s="117"/>
-      <c r="J7" s="117"/>
-      <c r="K7" s="118"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="102"/>
+      <c r="H7" s="102"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="103"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B8" s="116"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="117"/>
-      <c r="H8" s="117"/>
-      <c r="I8" s="117"/>
-      <c r="J8" s="117"/>
-      <c r="K8" s="118"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="102"/>
+      <c r="F8" s="102"/>
+      <c r="G8" s="102"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="102"/>
+      <c r="J8" s="102"/>
+      <c r="K8" s="103"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
-      <c r="F9" s="117"/>
-      <c r="G9" s="117"/>
-      <c r="H9" s="117"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="117"/>
-      <c r="K9" s="118"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="102"/>
+      <c r="H9" s="102"/>
+      <c r="I9" s="102"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="103"/>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B10" s="119"/>
-      <c r="C10" s="120"/>
-      <c r="D10" s="120"/>
-      <c r="E10" s="120"/>
-      <c r="F10" s="120"/>
-      <c r="G10" s="120"/>
-      <c r="H10" s="120"/>
-      <c r="I10" s="120"/>
-      <c r="J10" s="120"/>
-      <c r="K10" s="121"/>
+      <c r="B10" s="104"/>
+      <c r="C10" s="105"/>
+      <c r="D10" s="105"/>
+      <c r="E10" s="105"/>
+      <c r="F10" s="105"/>
+      <c r="G10" s="105"/>
+      <c r="H10" s="105"/>
+      <c r="I10" s="105"/>
+      <c r="J10" s="105"/>
+      <c r="K10" s="106"/>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B11" s="7"/>
@@ -6329,10 +6290,10 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" s="7"/>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="15"/>
+      <c r="D12" s="14"/>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
@@ -6346,7 +6307,7 @@
       <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="16"/>
+      <c r="D13" s="15"/>
       <c r="E13" s="4"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
@@ -6360,7 +6321,7 @@
       <c r="C14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="17">
+      <c r="D14" s="16">
         <v>500000</v>
       </c>
       <c r="E14" s="4"/>
@@ -6373,10 +6334,10 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B15" s="4"/>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="18" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="4"/>
@@ -6387,12 +6348,6 @@
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-    </row>
     <row r="17" spans="3:9" ht="17.25" x14ac:dyDescent="0.2">
       <c r="C17" s="1" t="s">
         <v>2</v>
@@ -6400,103 +6355,103 @@
       <c r="D17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="50" t="s">
+      <c r="E17" s="42" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C18" s="45">
+      <c r="C18" s="3">
         <v>0.25</v>
       </c>
-      <c r="D18" s="98">
+      <c r="D18" s="86">
         <v>0.02</v>
       </c>
-      <c r="E18" s="46">
+      <c r="E18" s="15">
         <f>1/(1+D18*C18)</f>
         <v>0.99502487562189068</v>
       </c>
-      <c r="F18" s="11"/>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C19" s="45">
+      <c r="C19" s="3">
         <v>0.5</v>
       </c>
-      <c r="D19" s="98">
+      <c r="D19" s="86">
         <v>2.4E-2</v>
       </c>
-      <c r="E19" s="46">
+      <c r="E19" s="15">
         <f t="shared" ref="E19:E21" si="0">1/(1+D19*C19)</f>
         <v>0.98814229249011853</v>
       </c>
     </row>
     <row r="20" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C20" s="45">
+      <c r="C20" s="3">
         <v>0.75</v>
       </c>
-      <c r="D20" s="98">
+      <c r="D20" s="86">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="15">
         <f t="shared" si="0"/>
         <v>0.97943192948090119</v>
       </c>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C21" s="45">
+      <c r="C21" s="3">
         <v>1</v>
       </c>
-      <c r="D21" s="98">
+      <c r="D21" s="86">
         <v>0.03</v>
       </c>
-      <c r="E21" s="46">
+      <c r="E21" s="15">
         <f t="shared" si="0"/>
         <v>0.970873786407767</v>
       </c>
     </row>
     <row r="22" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C22" s="47"/>
-      <c r="D22" s="39" t="s">
+      <c r="C22" s="17"/>
+      <c r="D22" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E22" s="40">
+      <c r="E22" s="35">
         <f>SUM(E18:E21)</f>
         <v>3.9334728840006772</v>
       </c>
     </row>
     <row r="24" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="D24" s="99" t="s">
+      <c r="D24" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="E24" s="41">
+      <c r="E24" s="36">
         <f>+(1-E21)/E22</f>
         <v>7.4047068458774155E-3</v>
       </c>
-      <c r="F24" s="35" t="s">
+      <c r="F24" s="31" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="25" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="D25" s="47" t="s">
+      <c r="D25" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E25" s="42">
+      <c r="E25" s="37">
         <f>+E24*4</f>
         <v>2.9618827383509662E-2</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="F25" s="25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C27" s="122" t="s">
+      <c r="C27" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="123"/>
-      <c r="E27" s="123"/>
-      <c r="F27" s="123"/>
-      <c r="G27" s="123"/>
-      <c r="H27" s="123"/>
-      <c r="I27" s="124"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="108"/>
+      <c r="F27" s="108"/>
+      <c r="G27" s="108"/>
+      <c r="H27" s="108"/>
+      <c r="I27" s="109"/>
     </row>
     <row r="29" spans="3:9" ht="17.25" x14ac:dyDescent="0.2">
       <c r="C29" s="1" t="s">
@@ -6505,79 +6460,79 @@
       <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="50" t="s">
+      <c r="E29" s="42" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C30" s="45">
+      <c r="C30" s="3">
         <v>0.25</v>
       </c>
-      <c r="D30" s="98">
+      <c r="D30" s="86">
         <v>0.03</v>
       </c>
-      <c r="E30" s="46">
+      <c r="E30" s="15">
         <f>1/(1+D30*C30)</f>
         <v>0.99255583126550861</v>
       </c>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C31" s="45">
+      <c r="C31" s="3">
         <v>0.5</v>
       </c>
-      <c r="D31" s="98">
+      <c r="D31" s="86">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="E31" s="46">
+      <c r="E31" s="15">
         <f t="shared" ref="E31:E32" si="1">1/(1+D31*C31)</f>
         <v>0.9837678307919332</v>
       </c>
     </row>
     <row r="32" spans="3:9" x14ac:dyDescent="0.2">
-      <c r="C32" s="45">
+      <c r="C32" s="3">
         <v>0.75</v>
       </c>
-      <c r="D32" s="98">
+      <c r="D32" s="86">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E32" s="46">
+      <c r="E32" s="15">
         <f t="shared" si="1"/>
         <v>0.97442143727161989</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C33" s="47"/>
-      <c r="D33" s="39" t="s">
+      <c r="C33" s="17"/>
+      <c r="D33" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E33" s="48">
+      <c r="E33" s="40">
         <f>SUM(E30:E32)</f>
         <v>2.9507450993290618</v>
       </c>
     </row>
     <row r="35" spans="3:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="D35" s="34" t="s">
+      <c r="D35" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E35" s="96">
+      <c r="E35" s="84">
         <f>+E24*D14*E33</f>
         <v>10924.701218720569</v>
       </c>
     </row>
     <row r="36" spans="3:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E36" s="97">
+      <c r="E36" s="85">
         <f>+D14*(1-E32)</f>
         <v>12789.281364190052</v>
       </c>
     </row>
     <row r="37" spans="3:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="D37" s="105" t="s">
+      <c r="D37" s="93" t="s">
         <v>97</v>
       </c>
-      <c r="E37" s="106">
+      <c r="E37" s="94">
         <f>+E36-E35</f>
         <v>1864.5801454694829</v>
       </c>
@@ -6604,502 +6559,466 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
-      <c r="E1" s="125"/>
-      <c r="F1" s="125"/>
-      <c r="G1" s="125"/>
-      <c r="H1" s="125"/>
-      <c r="I1" s="125"/>
-      <c r="J1" s="126"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="111"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="127"/>
-      <c r="C2" s="128"/>
-      <c r="D2" s="128"/>
-      <c r="E2" s="128"/>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="129"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="114"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B3" s="127"/>
-      <c r="C3" s="128"/>
-      <c r="D3" s="128"/>
-      <c r="E3" s="128"/>
-      <c r="F3" s="128"/>
-      <c r="G3" s="128"/>
-      <c r="H3" s="128"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="129"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="113"/>
+      <c r="I3" s="113"/>
+      <c r="J3" s="114"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="127"/>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128"/>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128"/>
-      <c r="G4" s="128"/>
-      <c r="H4" s="128"/>
-      <c r="I4" s="128"/>
-      <c r="J4" s="129"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="113"/>
+      <c r="I4" s="113"/>
+      <c r="J4" s="114"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B5" s="127"/>
-      <c r="C5" s="128"/>
-      <c r="D5" s="128"/>
-      <c r="E5" s="128"/>
-      <c r="F5" s="128"/>
-      <c r="G5" s="128"/>
-      <c r="H5" s="128"/>
-      <c r="I5" s="128"/>
-      <c r="J5" s="129"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="113"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="113"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="113"/>
+      <c r="J5" s="114"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B6" s="127"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="128"/>
-      <c r="E6" s="128"/>
-      <c r="F6" s="128"/>
-      <c r="G6" s="128"/>
-      <c r="H6" s="128"/>
-      <c r="I6" s="128"/>
-      <c r="J6" s="129"/>
+      <c r="B6" s="112"/>
+      <c r="C6" s="113"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="113"/>
+      <c r="G6" s="113"/>
+      <c r="H6" s="113"/>
+      <c r="I6" s="113"/>
+      <c r="J6" s="114"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="127"/>
-      <c r="C7" s="128"/>
-      <c r="D7" s="128"/>
-      <c r="E7" s="128"/>
-      <c r="F7" s="128"/>
-      <c r="G7" s="128"/>
-      <c r="H7" s="128"/>
-      <c r="I7" s="128"/>
-      <c r="J7" s="129"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="113"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="113"/>
+      <c r="H7" s="113"/>
+      <c r="I7" s="113"/>
+      <c r="J7" s="114"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="127"/>
-      <c r="C8" s="128"/>
-      <c r="D8" s="128"/>
-      <c r="E8" s="128"/>
-      <c r="F8" s="128"/>
-      <c r="G8" s="128"/>
-      <c r="H8" s="128"/>
-      <c r="I8" s="128"/>
-      <c r="J8" s="129"/>
+      <c r="B8" s="112"/>
+      <c r="C8" s="113"/>
+      <c r="D8" s="113"/>
+      <c r="E8" s="113"/>
+      <c r="F8" s="113"/>
+      <c r="G8" s="113"/>
+      <c r="H8" s="113"/>
+      <c r="I8" s="113"/>
+      <c r="J8" s="114"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="127"/>
-      <c r="C9" s="128"/>
-      <c r="D9" s="128"/>
-      <c r="E9" s="128"/>
-      <c r="F9" s="128"/>
-      <c r="G9" s="128"/>
-      <c r="H9" s="128"/>
-      <c r="I9" s="128"/>
-      <c r="J9" s="129"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="113"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="113"/>
+      <c r="F9" s="113"/>
+      <c r="G9" s="113"/>
+      <c r="H9" s="113"/>
+      <c r="I9" s="113"/>
+      <c r="J9" s="114"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B10" s="127"/>
-      <c r="C10" s="128"/>
-      <c r="D10" s="128"/>
-      <c r="E10" s="128"/>
-      <c r="F10" s="128"/>
-      <c r="G10" s="128"/>
-      <c r="H10" s="128"/>
-      <c r="I10" s="128"/>
-      <c r="J10" s="129"/>
+      <c r="B10" s="112"/>
+      <c r="C10" s="113"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="113"/>
+      <c r="F10" s="113"/>
+      <c r="G10" s="113"/>
+      <c r="H10" s="113"/>
+      <c r="I10" s="113"/>
+      <c r="J10" s="114"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="127"/>
-      <c r="C11" s="128"/>
-      <c r="D11" s="128"/>
-      <c r="E11" s="128"/>
-      <c r="F11" s="128"/>
-      <c r="G11" s="128"/>
-      <c r="H11" s="128"/>
-      <c r="I11" s="128"/>
-      <c r="J11" s="129"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="113"/>
+      <c r="G11" s="113"/>
+      <c r="H11" s="113"/>
+      <c r="I11" s="113"/>
+      <c r="J11" s="114"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="127"/>
-      <c r="C12" s="128"/>
-      <c r="D12" s="128"/>
-      <c r="E12" s="128"/>
-      <c r="F12" s="128"/>
-      <c r="G12" s="128"/>
-      <c r="H12" s="128"/>
-      <c r="I12" s="128"/>
-      <c r="J12" s="129"/>
+      <c r="B12" s="112"/>
+      <c r="C12" s="113"/>
+      <c r="D12" s="113"/>
+      <c r="E12" s="113"/>
+      <c r="F12" s="113"/>
+      <c r="G12" s="113"/>
+      <c r="H12" s="113"/>
+      <c r="I12" s="113"/>
+      <c r="J12" s="114"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="127"/>
-      <c r="C13" s="128"/>
-      <c r="D13" s="128"/>
-      <c r="E13" s="128"/>
-      <c r="F13" s="128"/>
-      <c r="G13" s="128"/>
-      <c r="H13" s="128"/>
-      <c r="I13" s="128"/>
-      <c r="J13" s="129"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="113"/>
+      <c r="D13" s="113"/>
+      <c r="E13" s="113"/>
+      <c r="F13" s="113"/>
+      <c r="G13" s="113"/>
+      <c r="H13" s="113"/>
+      <c r="I13" s="113"/>
+      <c r="J13" s="114"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="127"/>
-      <c r="C14" s="128"/>
-      <c r="D14" s="128"/>
-      <c r="E14" s="128"/>
-      <c r="F14" s="128"/>
-      <c r="G14" s="128"/>
-      <c r="H14" s="128"/>
-      <c r="I14" s="128"/>
-      <c r="J14" s="129"/>
+      <c r="B14" s="112"/>
+      <c r="C14" s="113"/>
+      <c r="D14" s="113"/>
+      <c r="E14" s="113"/>
+      <c r="F14" s="113"/>
+      <c r="G14" s="113"/>
+      <c r="H14" s="113"/>
+      <c r="I14" s="113"/>
+      <c r="J14" s="114"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B15" s="127"/>
-      <c r="C15" s="128"/>
-      <c r="D15" s="128"/>
-      <c r="E15" s="128"/>
-      <c r="F15" s="128"/>
-      <c r="G15" s="128"/>
-      <c r="H15" s="128"/>
-      <c r="I15" s="128"/>
-      <c r="J15" s="129"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="113"/>
+      <c r="E15" s="113"/>
+      <c r="F15" s="113"/>
+      <c r="G15" s="113"/>
+      <c r="H15" s="113"/>
+      <c r="I15" s="113"/>
+      <c r="J15" s="114"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B16" s="130"/>
-      <c r="C16" s="131"/>
-      <c r="D16" s="131"/>
-      <c r="E16" s="131"/>
-      <c r="F16" s="131"/>
-      <c r="G16" s="131"/>
-      <c r="H16" s="131"/>
-      <c r="I16" s="131"/>
-      <c r="J16" s="132"/>
+      <c r="B16" s="115"/>
+      <c r="C16" s="116"/>
+      <c r="D16" s="116"/>
+      <c r="E16" s="116"/>
+      <c r="F16" s="116"/>
+      <c r="G16" s="116"/>
+      <c r="H16" s="116"/>
+      <c r="I16" s="116"/>
+      <c r="J16" s="117"/>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C18" s="133" t="s">
+      <c r="C18" s="118" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="134"/>
-      <c r="E18" s="135"/>
+      <c r="D18" s="119"/>
+      <c r="E18" s="120"/>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="8">
         <v>5000000</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="22">
         <v>0.01</v>
       </c>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="24">
+      <c r="D21" s="6">
         <v>1</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="27" t="s">
+      <c r="D22" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="28"/>
-    </row>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="E22" s="25"/>
     </row>
     <row r="24" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C24" s="136" t="s">
+      <c r="C24" s="121" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="137"/>
-      <c r="E24" s="138"/>
+      <c r="D24" s="122"/>
+      <c r="E24" s="123"/>
     </row>
     <row r="25" spans="3:6" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D25" s="37" t="s">
+      <c r="D25" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="38" t="s">
+      <c r="E25" s="33" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C26" s="108">
+      <c r="C26" s="3">
         <v>0.5</v>
       </c>
       <c r="D26" s="5">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E26" s="109">
+      <c r="E26" s="15">
         <f t="shared" ref="E26:E27" si="0">1/(1+D26*C26)</f>
         <v>0.99850224663005482</v>
       </c>
     </row>
     <row r="27" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C27" s="108">
+      <c r="C27" s="3">
         <v>1</v>
       </c>
       <c r="D27" s="5">
         <v>3.8E-3</v>
       </c>
-      <c r="E27" s="109">
+      <c r="E27" s="15">
         <f t="shared" si="0"/>
         <v>0.99621438533572426</v>
       </c>
     </row>
     <row r="28" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C28" s="110"/>
-      <c r="D28" s="39" t="s">
+      <c r="C28" s="17"/>
+      <c r="D28" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E28" s="40">
+      <c r="E28" s="35">
         <f>SUM(E26:E27)</f>
         <v>1.9947166319657792</v>
       </c>
     </row>
     <row r="30" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="D30" s="99" t="s">
+      <c r="D30" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="41">
+      <c r="E30" s="36">
         <f>+(1-E27)/E28+E20</f>
         <v>1.1897820774946385E-2</v>
       </c>
-      <c r="F30" s="35" t="s">
+      <c r="F30" s="31" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="31" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="D31" s="47" t="s">
+      <c r="D31" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="42">
+      <c r="E31" s="37">
         <f>+E30*2</f>
         <v>2.379564154989277E-2</v>
       </c>
-      <c r="F31" s="28" t="s">
+      <c r="F31" s="25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="E32" s="12"/>
+      <c r="E32" s="11"/>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="C33" s="43" t="s">
+      <c r="C33" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="D33" s="100">
+      <c r="D33" s="88">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E33" s="80" t="s">
+      <c r="E33" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="F33" s="44"/>
+      <c r="F33" s="39"/>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B35" s="122" t="s">
+      <c r="B35" s="107" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="123"/>
-      <c r="D35" s="123"/>
-      <c r="E35" s="123"/>
-      <c r="F35" s="123"/>
-      <c r="G35" s="123"/>
-      <c r="H35" s="123"/>
-      <c r="I35" s="124"/>
+      <c r="C35" s="108"/>
+      <c r="D35" s="108"/>
+      <c r="E35" s="108"/>
+      <c r="F35" s="108"/>
+      <c r="G35" s="108"/>
+      <c r="H35" s="108"/>
+      <c r="I35" s="109"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="22"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="23"/>
+      <c r="B36" s="20"/>
+      <c r="I36" s="21"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="22"/>
-      <c r="C37" s="24" t="s">
+      <c r="B37" s="20"/>
+      <c r="C37" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D37" s="20">
+      <c r="D37" s="8">
         <f>+(D26*C26+E20)*D19</f>
         <v>57500</v>
       </c>
-      <c r="E37" s="24" t="s">
+      <c r="E37" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F37" s="29">
+      <c r="F37" s="26">
         <f>+D26*C26+E20</f>
         <v>1.15E-2</v>
       </c>
-      <c r="G37" s="24"/>
-      <c r="H37" s="24"/>
-      <c r="I37" s="23"/>
+      <c r="I37" s="21"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="22"/>
-      <c r="C38" s="24" t="s">
+      <c r="B38" s="20"/>
+      <c r="C38" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D38" s="20">
+      <c r="D38" s="8">
         <f>+(D33/2+E20)*D19</f>
         <v>62500</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="29">
-        <f>0.4%/2+E20</f>
-        <v>1.2E-2</v>
-      </c>
-      <c r="G38" s="24"/>
-      <c r="H38" s="24"/>
-      <c r="I38" s="23"/>
+      <c r="F38" s="26">
+        <f>D33/2+E20</f>
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="I38" s="21"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="26"/>
-      <c r="C39" s="30" t="s">
+      <c r="B39" s="23"/>
+      <c r="C39" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="31">
+      <c r="D39" s="28">
         <f>SUM(D37:D38)</f>
         <v>120000</v>
       </c>
-      <c r="E39" s="30" t="s">
+      <c r="E39" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="28"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="25"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B41" s="122" t="s">
+      <c r="B41" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="123"/>
-      <c r="D41" s="123"/>
-      <c r="E41" s="123"/>
-      <c r="F41" s="123"/>
-      <c r="G41" s="123"/>
-      <c r="H41" s="123"/>
-      <c r="I41" s="124"/>
+      <c r="C41" s="108"/>
+      <c r="D41" s="108"/>
+      <c r="E41" s="108"/>
+      <c r="F41" s="108"/>
+      <c r="G41" s="108"/>
+      <c r="H41" s="108"/>
+      <c r="I41" s="109"/>
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B42" s="22"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="24"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="23"/>
+      <c r="B42" s="20"/>
+      <c r="I42" s="21"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="22"/>
-      <c r="C43" s="24" t="s">
+      <c r="B43" s="20"/>
+      <c r="C43" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D43" s="20">
+      <c r="D43" s="8">
         <f>+E30*D19</f>
         <v>59489.103874731925</v>
       </c>
-      <c r="E43" s="24" t="s">
+      <c r="E43" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F43" s="29">
+      <c r="F43" s="26">
         <f>+E30</f>
         <v>1.1897820774946385E-2</v>
       </c>
-      <c r="G43" s="24"/>
-      <c r="H43" s="24"/>
-      <c r="I43" s="23"/>
+      <c r="I43" s="21"/>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="22"/>
-      <c r="C44" s="32" t="s">
+      <c r="B44" s="20"/>
+      <c r="C44" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D44" s="21">
+      <c r="D44" s="19">
         <f>+D43*2</f>
         <v>118978.20774946385</v>
       </c>
-      <c r="E44" s="32" t="s">
+      <c r="E44" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F44" s="24"/>
-      <c r="G44" s="24"/>
-      <c r="H44" s="24"/>
-      <c r="I44" s="23"/>
+      <c r="I44" s="21"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="22"/>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="24"/>
-      <c r="H45" s="24"/>
-      <c r="I45" s="23"/>
+      <c r="B45" s="20"/>
+      <c r="I45" s="21"/>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B46" s="22"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="33">
+      <c r="B46" s="20"/>
+      <c r="D46" s="29">
         <f>+D39-D44</f>
         <v>1021.7922505361494</v>
       </c>
-      <c r="E46" s="32" t="s">
+      <c r="E46" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F46" s="24"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="23"/>
+      <c r="I46" s="21"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B47" s="26"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="27" t="s">
+      <c r="B47" s="23"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="28"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="24"/>
+      <c r="I47" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7130,94 +7049,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="115"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" s="116"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="118"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="103"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="118"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="118"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="103"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="118"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="103"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="116"/>
-      <c r="C6" s="117"/>
-      <c r="D6" s="117"/>
-      <c r="E6" s="117"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="118"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="103"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="116"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="118"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="103"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="116"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="102"/>
+      <c r="F8" s="102"/>
+      <c r="G8" s="103"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
-      <c r="F9" s="117"/>
-      <c r="G9" s="118"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="103"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="116"/>
-      <c r="C10" s="117"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="117"/>
-      <c r="G10" s="118"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="103"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="119"/>
-      <c r="C11" s="120"/>
-      <c r="D11" s="120"/>
-      <c r="E11" s="120"/>
-      <c r="F11" s="120"/>
-      <c r="G11" s="121"/>
+      <c r="B11" s="104"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="105"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="106"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="7"/>
@@ -7228,123 +7147,120 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="57">
+      <c r="C13" s="47">
         <v>10</v>
       </c>
-      <c r="D13" s="35" t="s">
+      <c r="D13" s="31" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="23"/>
+      <c r="D14" s="21"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="58">
+      <c r="C15" s="48">
         <v>0.05</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="21" t="s">
         <v>44</v>
       </c>
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="8">
         <v>3500000000</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="49"/>
+      <c r="E16" s="41"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="58">
+      <c r="C17" s="48">
         <v>0.02</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="21" t="s">
         <v>44</v>
       </c>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="55">
+      <c r="C18" s="45">
         <v>1000000</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="25" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="8"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="35"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="31"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="8">
         <v>3600</v>
       </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="23"/>
+      <c r="E21" s="21"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B22" s="22"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="23"/>
+      <c r="B22" s="20"/>
+      <c r="E22" s="21"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="58">
+      <c r="C23" s="48">
         <v>0.05</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="G23" s="20"/>
+      <c r="G23" s="8"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="59">
+      <c r="C24" s="49">
         <v>0.02</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="28" t="s">
+      <c r="E24" s="25" t="s">
         <v>40</v>
       </c>
     </row>
@@ -7359,28 +7275,28 @@
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
-      <c r="H26" s="50"/>
+      <c r="H26" s="42"/>
     </row>
     <row r="27" spans="2:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="37" t="s">
+      <c r="C27" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="37" t="s">
+      <c r="D27" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E27" s="37" t="s">
+      <c r="E27" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F27" s="37" t="s">
+      <c r="F27" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G27" s="37" t="s">
+      <c r="G27" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="H27" s="38" t="s">
+      <c r="H27" s="33" t="s">
         <v>50</v>
       </c>
     </row>
@@ -7388,26 +7304,26 @@
       <c r="B28" s="3">
         <v>6</v>
       </c>
-      <c r="C28" s="52">
+      <c r="C28" s="4">
         <v>0</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="8">
         <f>+$C$15*$C$16</f>
         <v>175000000</v>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="8">
         <f>+$C$17*$C$18</f>
         <v>20000</v>
       </c>
-      <c r="F28" s="53">
+      <c r="F28" s="41">
         <f>+C21</f>
         <v>3600</v>
       </c>
-      <c r="G28" s="20">
+      <c r="G28" s="8">
         <f>+D28-E28*F28</f>
         <v>103000000</v>
       </c>
-      <c r="H28" s="17">
+      <c r="H28" s="16">
         <f>+G28</f>
         <v>103000000</v>
       </c>
@@ -7416,26 +7332,26 @@
       <c r="B29" s="3">
         <v>7</v>
       </c>
-      <c r="C29" s="52">
+      <c r="C29" s="4">
         <v>1</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="8">
         <f>+$C$15*$C$16</f>
         <v>175000000</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="8">
         <f>+$C$17*$C$18</f>
         <v>20000</v>
       </c>
-      <c r="F29" s="53">
+      <c r="F29" s="41">
         <f>+$C$21*((1+$C$23)/(1+$C$24))^C29</f>
         <v>3705.882352941177</v>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="8">
         <f t="shared" ref="G29:G32" si="0">+D29-E29*F29</f>
         <v>100882352.94117646</v>
       </c>
-      <c r="H29" s="17">
+      <c r="H29" s="16">
         <f>+G29/(1+$C$23)^C29</f>
         <v>96078431.372548997</v>
       </c>
@@ -7444,26 +7360,26 @@
       <c r="B30" s="3">
         <v>8</v>
       </c>
-      <c r="C30" s="52">
+      <c r="C30" s="4">
         <v>2</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="8">
         <f t="shared" ref="D30:D31" si="1">+$C$15*$C$16</f>
         <v>175000000</v>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="8">
         <f t="shared" ref="E30:E31" si="2">+$C$17*$C$18</f>
         <v>20000</v>
       </c>
-      <c r="F30" s="53">
+      <c r="F30" s="41">
         <f t="shared" ref="F30:F32" si="3">+$C$21*((1+$C$23)/(1+$C$24))^C30</f>
         <v>3814.8788927335645</v>
       </c>
-      <c r="G30" s="20">
+      <c r="G30" s="8">
         <f t="shared" si="0"/>
         <v>98702422.145328715</v>
       </c>
-      <c r="H30" s="17">
+      <c r="H30" s="16">
         <f t="shared" ref="H30:H32" si="4">+G30/(1+$C$23)^C30</f>
         <v>89526006.481023774</v>
       </c>
@@ -7472,26 +7388,26 @@
       <c r="B31" s="3">
         <v>9</v>
       </c>
-      <c r="C31" s="52">
+      <c r="C31" s="4">
         <v>3</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="8">
         <f t="shared" si="1"/>
         <v>175000000</v>
       </c>
-      <c r="E31" s="20">
+      <c r="E31" s="8">
         <f t="shared" si="2"/>
         <v>20000</v>
       </c>
-      <c r="F31" s="53">
+      <c r="F31" s="41">
         <f t="shared" si="3"/>
         <v>3927.0812131080816</v>
       </c>
-      <c r="G31" s="20">
+      <c r="G31" s="8">
         <f t="shared" si="0"/>
         <v>96458375.737838373</v>
       </c>
-      <c r="H31" s="17">
+      <c r="H31" s="16">
         <f t="shared" si="4"/>
         <v>83324371.655621082</v>
       </c>
@@ -7500,44 +7416,44 @@
       <c r="B32" s="3">
         <v>10</v>
       </c>
-      <c r="C32" s="52">
+      <c r="C32" s="4">
         <v>4</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="8">
         <f>+$C$15*$C$16+C16</f>
         <v>3675000000</v>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="8">
         <f>+$C$17*$C$18+C18</f>
         <v>1020000</v>
       </c>
-      <c r="F32" s="53">
+      <c r="F32" s="41">
         <f t="shared" si="3"/>
         <v>4042.583601728908</v>
       </c>
-      <c r="G32" s="20">
+      <c r="G32" s="8">
         <f t="shared" si="0"/>
         <v>-448435273.76348591</v>
       </c>
-      <c r="H32" s="17">
+      <c r="H32" s="16">
         <f t="shared" si="4"/>
         <v>-368928809.50919497</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="B33" s="18"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="54"/>
-      <c r="G33" s="39" t="s">
+      <c r="B33" s="17"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="H33" s="56">
+      <c r="H33" s="46">
         <f>SUM(H28:H32)</f>
         <v>2999999.9999989271</v>
       </c>
-      <c r="I33" s="13"/>
+      <c r="I33" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7561,161 +7477,161 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="115"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" s="116"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="118"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="103"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="118"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="103"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="118"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="103"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="118"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="103"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="116"/>
-      <c r="C6" s="117"/>
-      <c r="D6" s="117"/>
-      <c r="E6" s="117"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="118"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="103"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="116"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="118"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="103"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="116"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="118"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="102"/>
+      <c r="F8" s="102"/>
+      <c r="G8" s="103"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
-      <c r="F9" s="117"/>
-      <c r="G9" s="118"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="103"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="116"/>
-      <c r="C10" s="117"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="117"/>
-      <c r="G10" s="118"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="103"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="119"/>
-      <c r="C11" s="120"/>
-      <c r="D11" s="120"/>
-      <c r="E11" s="120"/>
-      <c r="F11" s="120"/>
-      <c r="G11" s="121"/>
+      <c r="B11" s="104"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="105"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="106"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="104">
+      <c r="C14" s="92">
         <v>0.03</v>
       </c>
-      <c r="D14" s="35" t="s">
+      <c r="D14" s="31" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="52" t="s">
+      <c r="C15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="23"/>
+      <c r="D15" s="21"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="8">
         <v>5000000</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="52">
+      <c r="C17" s="4">
         <v>5</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="21" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="54" t="s">
+      <c r="C18" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="28"/>
+      <c r="D18" s="25"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="57"/>
-      <c r="D21" s="35"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="31"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="59">
+      <c r="C22" s="49">
         <v>0.03</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="25" t="s">
         <v>63</v>
       </c>
       <c r="E22" s="6" t="s">
@@ -7723,13 +7639,13 @@
       </c>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="63">
+      <c r="C24" s="51">
         <v>0.02</v>
       </c>
-      <c r="D24" s="44" t="s">
+      <c r="D24" s="39" t="s">
         <v>63</v>
       </c>
       <c r="E24" s="6" t="s">
@@ -7745,26 +7661,26 @@
       <c r="E26" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="35"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="31"/>
     </row>
     <row r="27" spans="2:8" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="37" t="s">
+      <c r="C27" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="37" t="s">
+      <c r="D27" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="37" t="s">
+      <c r="E27" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F27" s="60" t="s">
+      <c r="F27" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="G27" s="61" t="s">
+      <c r="G27" s="33" t="s">
         <v>61</v>
       </c>
     </row>
@@ -7772,140 +7688,140 @@
       <c r="B28" s="3">
         <v>3</v>
       </c>
-      <c r="C28" s="52">
+      <c r="C28" s="4">
         <v>0</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="8">
         <f>+$C$14/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="8">
         <f>+C24/2*C16</f>
         <v>50000</v>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="8">
         <f>+D28-E28</f>
         <v>25000</v>
       </c>
-      <c r="G28" s="17">
+      <c r="G28" s="16">
         <f>+F28/(1+$C$22/2)^C28</f>
         <v>25000</v>
       </c>
-      <c r="H28" s="20"/>
+      <c r="H28" s="8"/>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B29" s="3">
         <v>3.5</v>
       </c>
-      <c r="C29" s="52">
+      <c r="C29" s="4">
         <v>1</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="8">
         <f>+$C$14/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="8">
         <f>+$C$22/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="8">
         <f t="shared" ref="F29:F32" si="0">+D29-E29</f>
         <v>0</v>
       </c>
-      <c r="G29" s="17">
+      <c r="G29" s="16">
         <f>+F29/(1+$C$22/2)^C29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="20"/>
+      <c r="H29" s="8"/>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B30" s="3">
         <v>4</v>
       </c>
-      <c r="C30" s="52">
+      <c r="C30" s="4">
         <v>2</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="8">
         <f>+$C$14/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="8">
         <f>+$C$22/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="F30" s="20">
+      <c r="F30" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G30" s="17">
+      <c r="G30" s="16">
         <f t="shared" ref="G30:G32" si="1">+F30/(1+$C$22/2)^C30</f>
         <v>0</v>
       </c>
-      <c r="H30" s="20"/>
+      <c r="H30" s="8"/>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B31" s="3">
         <v>4.5</v>
       </c>
-      <c r="C31" s="52">
+      <c r="C31" s="4">
         <v>3</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="8">
         <f>+$C$14/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="E31" s="20">
+      <c r="E31" s="8">
         <f>+$C$22/2*$C$16</f>
         <v>75000</v>
       </c>
-      <c r="F31" s="20">
+      <c r="F31" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G31" s="17">
+      <c r="G31" s="16">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H31" s="20"/>
+      <c r="H31" s="8"/>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B32" s="3">
         <v>5</v>
       </c>
-      <c r="C32" s="52">
+      <c r="C32" s="4">
         <v>4</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="8">
         <f>+$C$14/2*$C$16+C16</f>
         <v>5075000</v>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="8">
         <f>+$C$22/2*$C$16+C16</f>
         <v>5075000</v>
       </c>
-      <c r="F32" s="20">
+      <c r="F32" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="16">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H32" s="20"/>
+      <c r="H32" s="8"/>
     </row>
     <row r="33" spans="2:8" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="B33" s="18"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="31" t="s">
+      <c r="B33" s="17"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="G33" s="56">
+      <c r="G33" s="46">
         <f>SUM(G28:G32)</f>
         <v>25000</v>
       </c>
-      <c r="H33" s="20"/>
+      <c r="H33" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7933,342 +7849,342 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B2" s="116"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="118"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="103"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B6" s="116"/>
-      <c r="C6" s="117"/>
-      <c r="D6" s="117"/>
-      <c r="E6" s="118"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
-      <c r="H6" s="67"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="116"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="118"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="67"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="103"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="55"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B8" s="116"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="118"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
-      <c r="H8" s="67"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="103"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="118"/>
-      <c r="F9" s="67"/>
-      <c r="G9" s="67"/>
-      <c r="H9" s="67"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="103"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B10" s="116"/>
-      <c r="C10" s="117"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="118"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="67"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="103"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B11" s="119"/>
-      <c r="C11" s="120"/>
-      <c r="D11" s="120"/>
-      <c r="E11" s="121"/>
-      <c r="F11" s="67"/>
-      <c r="G11" s="67"/>
-      <c r="H11" s="67"/>
+      <c r="B11" s="104"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="106"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="55"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="70">
+      <c r="C12" s="58">
         <v>0.04</v>
       </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="67"/>
-      <c r="F12" s="67"/>
-      <c r="G12" s="67"/>
-      <c r="H12" s="67"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="71">
+      <c r="C13" s="59">
         <v>0.06</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="67"/>
-      <c r="F13" s="67"/>
-      <c r="G13" s="67"/>
-      <c r="H13" s="67"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="28"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="67"/>
-      <c r="G14" s="67"/>
-      <c r="H14" s="67"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B15" s="67"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="55"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="101">
+      <c r="C16" s="89">
         <v>1000000000</v>
       </c>
-      <c r="D16" s="72"/>
+      <c r="D16" s="60"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="8">
         <v>10000000</v>
       </c>
-      <c r="D17" s="73"/>
+      <c r="D17" s="61"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C18" s="52">
+      <c r="C18" s="4">
         <v>2</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="21" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="52">
+      <c r="C19" s="4">
         <v>115</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="21" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="74">
+      <c r="C20" s="62">
         <f>1/C19</f>
         <v>8.6956521739130436E-3</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="25" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B22" s="133" t="s">
+      <c r="B22" s="118" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="135"/>
-      <c r="E22" s="133" t="s">
+      <c r="C22" s="120"/>
+      <c r="E22" s="118" t="s">
         <v>77</v>
       </c>
-      <c r="F22" s="135"/>
+      <c r="F22" s="120"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="46" t="s">
+      <c r="C23" s="15" t="s">
         <v>76</v>
       </c>
       <c r="D23" s="4"/>
-      <c r="E23" s="45" t="s">
+      <c r="E23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="46" t="s">
+      <c r="F23" s="15" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B24" s="45">
+      <c r="B24" s="3">
         <v>1</v>
       </c>
-      <c r="C24" s="75">
+      <c r="C24" s="63">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="D24" s="4"/>
-      <c r="E24" s="45">
+      <c r="E24" s="3">
         <v>1</v>
       </c>
-      <c r="F24" s="75">
+      <c r="F24" s="63">
         <v>0.02</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B25" s="47">
+      <c r="B25" s="17">
         <v>2</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="64">
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="D25" s="4"/>
-      <c r="E25" s="47">
+      <c r="E25" s="17">
         <v>2</v>
       </c>
-      <c r="F25" s="76">
+      <c r="F25" s="64">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="4"/>
-      <c r="C26" s="65"/>
+      <c r="C26" s="53"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
-      <c r="F26" s="65"/>
+      <c r="F26" s="53"/>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="77" t="s">
+      <c r="C27" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B28" s="36">
+      <c r="B28" s="32">
         <v>1</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="8">
         <f>+$C$13*$C$17</f>
         <v>600000</v>
       </c>
-      <c r="D28" s="17">
+      <c r="D28" s="16">
         <f>+C28*EXP(-F24*B28)</f>
         <v>588119.20398405311</v>
       </c>
-      <c r="E28" s="64"/>
-      <c r="F28" s="66"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="54"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B29" s="36">
+      <c r="B29" s="32">
         <v>2</v>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="8">
         <f>+$C$13*$C$17+C17</f>
         <v>10600000</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="16">
         <f>+C29*EXP(-F25*B29)</f>
         <v>10083031.899707569</v>
       </c>
-      <c r="E29" s="64"/>
-      <c r="F29" s="66"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="54"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B30" s="47"/>
-      <c r="C30" s="78" t="s">
+      <c r="B30" s="17"/>
+      <c r="C30" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="79">
+      <c r="D30" s="67">
         <f>SUM(D28:D29)</f>
         <v>10671151.103691623</v>
       </c>
       <c r="E30" s="4"/>
-      <c r="F30" s="66"/>
+      <c r="F30" s="54"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="4"/>
-      <c r="C31" s="65"/>
-      <c r="D31" s="66"/>
+      <c r="C31" s="53"/>
+      <c r="D31" s="54"/>
       <c r="E31" s="4"/>
-      <c r="F31" s="66"/>
+      <c r="F31" s="54"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="77" t="s">
+      <c r="C32" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="50" t="s">
+      <c r="D32" s="42" t="s">
         <v>80</v>
       </c>
       <c r="E32" s="1" t="s">
@@ -8277,105 +8193,105 @@
       <c r="F32" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G32" s="50" t="s">
+      <c r="G32" s="42" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="36">
+      <c r="B33" s="32">
         <v>1</v>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="8">
         <f>+C12*C16</f>
         <v>40000000</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="16">
         <f>+C33*EXP(-C24*B33)</f>
         <v>39800499.167707294</v>
       </c>
-      <c r="E33" s="45">
+      <c r="E33" s="3">
         <f>+$C$20*EXP((F24-C24)*B33)</f>
         <v>8.8270701270932086E-3</v>
       </c>
-      <c r="F33" s="20">
+      <c r="F33" s="8">
         <f>+E33*C33</f>
         <v>353082.80508372834</v>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="16">
         <f>+F33*EXP(-F24*B33)</f>
         <v>346091.29711049818</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="36">
+      <c r="B34" s="32">
         <v>2</v>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="8">
         <f>+C12*C16+C16</f>
         <v>1040000000</v>
       </c>
-      <c r="D34" s="17">
+      <c r="D34" s="16">
         <f>+C34*EXP(-C25*B34)</f>
         <v>1023492412.8574965</v>
       </c>
-      <c r="E34" s="45">
+      <c r="E34" s="3">
         <f>+$C$20*EXP((F25-C25)*B34)</f>
         <v>8.9963878845923297E-3</v>
       </c>
-      <c r="F34" s="20">
+      <c r="F34" s="8">
         <f>+E34*C34</f>
         <v>9356243.3999760225</v>
       </c>
-      <c r="G34" s="17">
+      <c r="G34" s="16">
         <f>+F34*EXP(-F25*B34)</f>
         <v>8899934.0248477962</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B35" s="47"/>
-      <c r="C35" s="78" t="s">
+      <c r="B35" s="17"/>
+      <c r="C35" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="56">
+      <c r="D35" s="46">
         <f>SUM(D33:D34)</f>
         <v>1063292912.0252038</v>
       </c>
-      <c r="E35" s="102"/>
-      <c r="F35" s="78" t="s">
+      <c r="E35" s="90"/>
+      <c r="F35" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="G35" s="56">
+      <c r="G35" s="46">
         <f>SUM(G33:G34)</f>
         <v>9246025.3219582941</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B36" s="4"/>
-      <c r="C36" s="65"/>
+      <c r="C36" s="53"/>
       <c r="E36" s="4"/>
-      <c r="F36" s="65"/>
-      <c r="I36" s="103"/>
+      <c r="F36" s="53"/>
+      <c r="I36" s="91"/>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B37" s="4"/>
-      <c r="D37" s="66"/>
+      <c r="D37" s="54"/>
       <c r="E37" s="4"/>
-      <c r="F37" s="65"/>
+      <c r="F37" s="53"/>
     </row>
     <row r="38" spans="2:9" ht="17.25" x14ac:dyDescent="0.2">
       <c r="B38" s="4"/>
-      <c r="C38" s="68" t="s">
+      <c r="C38" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="D38" s="69">
+      <c r="D38" s="57">
         <f>+D35*C20-D30</f>
         <v>-1425125.7817333285</v>
       </c>
       <c r="E38" s="4"/>
-      <c r="F38" s="68" t="s">
+      <c r="F38" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="G38" s="69">
+      <c r="G38" s="57">
         <f>+G35-D30</f>
         <v>-1425125.7817333285</v>
       </c>
@@ -8393,7 +8309,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702B449C-4594-422A-8A06-A774A1918956}">
-  <dimension ref="B1:J58"/>
+  <dimension ref="B1:J57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="11.42578125" style="6"/>
@@ -8407,374 +8323,374 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="98" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
-      <c r="F1" s="114"/>
-      <c r="G1" s="114"/>
-      <c r="H1" s="114"/>
-      <c r="I1" s="114"/>
-      <c r="J1" s="115"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="100"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="116"/>
-      <c r="C2" s="117"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="117"/>
-      <c r="H2" s="117"/>
-      <c r="I2" s="117"/>
-      <c r="J2" s="118"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="103"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B3" s="116"/>
-      <c r="C3" s="117"/>
-      <c r="D3" s="117"/>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="117"/>
-      <c r="H3" s="117"/>
-      <c r="I3" s="117"/>
-      <c r="J3" s="118"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="103"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B4" s="116"/>
-      <c r="C4" s="117"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="118"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="103"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="117"/>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="117"/>
-      <c r="H5" s="117"/>
-      <c r="I5" s="117"/>
-      <c r="J5" s="118"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="102"/>
+      <c r="G5" s="102"/>
+      <c r="H5" s="102"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="103"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B6" s="116"/>
-      <c r="C6" s="117"/>
-      <c r="D6" s="117"/>
-      <c r="E6" s="117"/>
-      <c r="F6" s="117"/>
-      <c r="G6" s="117"/>
-      <c r="H6" s="117"/>
-      <c r="I6" s="117"/>
-      <c r="J6" s="118"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="102"/>
+      <c r="J6" s="103"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B7" s="116"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="117"/>
-      <c r="E7" s="117"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="117"/>
-      <c r="H7" s="117"/>
-      <c r="I7" s="117"/>
-      <c r="J7" s="118"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="102"/>
+      <c r="H7" s="102"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="103"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B8" s="116"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="117"/>
-      <c r="E8" s="117"/>
-      <c r="F8" s="117"/>
-      <c r="G8" s="117"/>
-      <c r="H8" s="117"/>
-      <c r="I8" s="117"/>
-      <c r="J8" s="118"/>
+      <c r="B8" s="101"/>
+      <c r="C8" s="102"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="102"/>
+      <c r="F8" s="102"/>
+      <c r="G8" s="102"/>
+      <c r="H8" s="102"/>
+      <c r="I8" s="102"/>
+      <c r="J8" s="103"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
-      <c r="F9" s="117"/>
-      <c r="G9" s="117"/>
-      <c r="H9" s="117"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="118"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="102"/>
+      <c r="H9" s="102"/>
+      <c r="I9" s="102"/>
+      <c r="J9" s="103"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B10" s="116"/>
-      <c r="C10" s="117"/>
-      <c r="D10" s="117"/>
-      <c r="E10" s="117"/>
-      <c r="F10" s="117"/>
-      <c r="G10" s="117"/>
-      <c r="H10" s="117"/>
-      <c r="I10" s="117"/>
-      <c r="J10" s="118"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="102"/>
+      <c r="H10" s="102"/>
+      <c r="I10" s="102"/>
+      <c r="J10" s="103"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B11" s="116"/>
-      <c r="C11" s="117"/>
-      <c r="D11" s="117"/>
-      <c r="E11" s="117"/>
-      <c r="F11" s="117"/>
-      <c r="G11" s="117"/>
-      <c r="H11" s="117"/>
-      <c r="I11" s="117"/>
-      <c r="J11" s="118"/>
+      <c r="B11" s="101"/>
+      <c r="C11" s="102"/>
+      <c r="D11" s="102"/>
+      <c r="E11" s="102"/>
+      <c r="F11" s="102"/>
+      <c r="G11" s="102"/>
+      <c r="H11" s="102"/>
+      <c r="I11" s="102"/>
+      <c r="J11" s="103"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B12" s="116"/>
-      <c r="C12" s="117"/>
-      <c r="D12" s="117"/>
-      <c r="E12" s="117"/>
-      <c r="F12" s="117"/>
-      <c r="G12" s="117"/>
-      <c r="H12" s="117"/>
-      <c r="I12" s="117"/>
-      <c r="J12" s="118"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="102"/>
+      <c r="D12" s="102"/>
+      <c r="E12" s="102"/>
+      <c r="F12" s="102"/>
+      <c r="G12" s="102"/>
+      <c r="H12" s="102"/>
+      <c r="I12" s="102"/>
+      <c r="J12" s="103"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="119"/>
-      <c r="C13" s="120"/>
-      <c r="D13" s="120"/>
-      <c r="E13" s="120"/>
-      <c r="F13" s="120"/>
-      <c r="G13" s="120"/>
-      <c r="H13" s="120"/>
-      <c r="I13" s="120"/>
-      <c r="J13" s="121"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="105"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="105"/>
+      <c r="G13" s="105"/>
+      <c r="H13" s="105"/>
+      <c r="I13" s="105"/>
+      <c r="J13" s="106"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="C15" s="133" t="s">
+      <c r="C15" s="118" t="s">
         <v>82</v>
       </c>
-      <c r="D15" s="134"/>
-      <c r="E15" s="135"/>
+      <c r="D15" s="119"/>
+      <c r="E15" s="120"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="8">
         <v>10000000</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D17" s="81" t="s">
+      <c r="D17" s="69" t="s">
         <v>96</v>
       </c>
-      <c r="E17" s="23"/>
+      <c r="E17" s="21"/>
     </row>
     <row r="18" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C18" s="26" t="s">
+      <c r="C18" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="85">
+      <c r="D18" s="73">
         <v>5</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="25" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C22" s="136" t="s">
+      <c r="C22" s="121" t="s">
         <v>85</v>
       </c>
-      <c r="D22" s="137"/>
-      <c r="E22" s="112"/>
-      <c r="G22" s="136" t="s">
+      <c r="D22" s="122"/>
+      <c r="E22" s="97"/>
+      <c r="G22" s="121" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="137"/>
-      <c r="I22" s="111"/>
-      <c r="J22" s="112"/>
+      <c r="H22" s="122"/>
+      <c r="I22" s="96"/>
+      <c r="J22" s="97"/>
     </row>
     <row r="23" spans="3:10" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="C23" s="36" t="s">
+      <c r="C23" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="D23" s="37" t="s">
+      <c r="D23" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="38" t="s">
+      <c r="E23" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="G23" s="36" t="s">
+      <c r="G23" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="H23" s="37" t="s">
+      <c r="H23" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="I23" s="37" t="s">
+      <c r="I23" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="J23" s="38" t="s">
+      <c r="J23" s="33" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C24" s="45">
+      <c r="C24" s="3">
         <v>3</v>
       </c>
       <c r="D24" s="5">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="E24" s="46">
+      <c r="E24" s="15">
         <f>1/(1+D24*C24/12)</f>
         <v>0.99378881987577627</v>
       </c>
-      <c r="G24" s="45">
+      <c r="G24" s="3">
         <v>3</v>
       </c>
       <c r="H24" s="5">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="I24" s="52">
+      <c r="I24" s="4">
         <f>1/(1+H24*G24/12)</f>
         <v>0.99920063948840931</v>
       </c>
-      <c r="J24" s="93">
+      <c r="J24" s="81">
         <f>+H24</f>
         <v>3.2000000000000002E-3</v>
       </c>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C25" s="45">
+      <c r="C25" s="3">
         <f>+C24+3</f>
         <v>6</v>
       </c>
       <c r="D25" s="5">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="E25" s="46">
+      <c r="E25" s="15">
         <f t="shared" ref="E25:E27" si="0">1/(1+D25*C25/12)</f>
         <v>0.98619329388560162</v>
       </c>
-      <c r="G25" s="45">
+      <c r="G25" s="3">
         <f>+G24+3</f>
         <v>6</v>
       </c>
       <c r="H25" s="5">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="I25" s="52">
+      <c r="I25" s="4">
         <f t="shared" ref="I25:I27" si="1">1/(1+H25*G25/12)</f>
         <v>0.99825305714998758</v>
       </c>
-      <c r="J25" s="93">
+      <c r="J25" s="81">
         <f>+((1+H25*G25/12)/(1+H24*G24/12)-1)*12/(G25-G24)</f>
         <v>3.7969624300560056E-3</v>
       </c>
     </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C26" s="45">
+      <c r="C26" s="3">
         <f>+C25+3</f>
         <v>9</v>
       </c>
       <c r="D26" s="5">
         <v>3.1E-2</v>
       </c>
-      <c r="E26" s="46">
+      <c r="E26" s="15">
         <f t="shared" si="0"/>
         <v>0.97727827999022721</v>
       </c>
-      <c r="G26" s="45">
+      <c r="G26" s="3">
         <f>+G25+3</f>
         <v>9</v>
       </c>
       <c r="H26" s="5">
         <v>3.8E-3</v>
       </c>
-      <c r="I26" s="52">
+      <c r="I26" s="4">
         <f t="shared" si="1"/>
         <v>0.99715809941666245</v>
       </c>
-      <c r="J26" s="93">
+      <c r="J26" s="81">
         <f t="shared" ref="J26" si="2">+((1+H26*G26/12)/(1+H25*G25/12)-1)*12/(G26-G25)</f>
         <v>4.3923134514605167E-3</v>
       </c>
     </row>
     <row r="27" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C27" s="45">
+      <c r="C27" s="3">
         <f t="shared" ref="C27" si="3">+C26+3</f>
         <v>12</v>
       </c>
       <c r="D27" s="5">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E27" s="46">
+      <c r="E27" s="15">
         <f t="shared" si="0"/>
         <v>0.96618357487922713</v>
       </c>
-      <c r="G27" s="45">
+      <c r="G27" s="3">
         <f t="shared" ref="G27" si="4">+G26+3</f>
         <v>12</v>
       </c>
       <c r="H27" s="5">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="I27" s="52">
+      <c r="I27" s="4">
         <f t="shared" si="1"/>
         <v>0.99601593625498008</v>
       </c>
-      <c r="J27" s="93">
+      <c r="J27" s="81">
         <f>+((1+H27*G27/12)/(1+H26*G26/12)-1)*12/(G27-G26)</f>
         <v>4.5869272573169084E-3</v>
       </c>
     </row>
     <row r="28" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C28" s="47"/>
-      <c r="D28" s="39" t="s">
+      <c r="C28" s="17"/>
+      <c r="D28" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="E28" s="40">
+      <c r="E28" s="35">
         <f>SUM(E24:E27)</f>
         <v>3.9234439686308322</v>
       </c>
-      <c r="G28" s="26"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="28"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="25"/>
     </row>
     <row r="29" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C29" s="4"/>
     </row>
     <row r="30" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C30" s="4"/>
-      <c r="D30" s="94" t="s">
+      <c r="D30" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="95">
+      <c r="E30" s="83">
         <f>+(1-E27)/E28</f>
         <v>8.6190666646818008E-3</v>
       </c>
-      <c r="F30" s="44" t="s">
+      <c r="F30" s="39" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="31" spans="3:10" x14ac:dyDescent="0.2">
       <c r="C31" s="4"/>
-      <c r="D31" s="94" t="s">
+      <c r="D31" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="95">
+      <c r="E31" s="83">
         <f>+E30*4</f>
         <v>3.4476266658727203E-2</v>
       </c>
-      <c r="F31" s="44" t="s">
+      <c r="F31" s="39" t="s">
         <v>5</v>
       </c>
     </row>
@@ -8782,170 +8698,167 @@
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C33" s="139" t="s">
+      <c r="C33" s="124" t="s">
         <v>89</v>
       </c>
-      <c r="D33" s="140"/>
-      <c r="E33" s="141"/>
+      <c r="D33" s="125"/>
+      <c r="E33" s="126"/>
     </row>
     <row r="34" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C34" s="82" t="s">
+      <c r="C34" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="D34" s="81" t="s">
+      <c r="D34" s="69" t="s">
         <v>96</v>
       </c>
-      <c r="E34" s="23" t="s">
+      <c r="E34" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="F34" s="11"/>
+      <c r="F34" s="10"/>
     </row>
     <row r="35" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C35" s="82" t="s">
+      <c r="C35" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="D35" s="62">
+      <c r="D35" s="50">
         <f>+D16</f>
         <v>10000000</v>
       </c>
-      <c r="E35" s="23" t="s">
+      <c r="E35" s="21" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="36" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C36" s="82" t="s">
+      <c r="C36" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="89">
+      <c r="D36" s="77">
         <f>+E30</f>
         <v>8.6190666646818008E-3</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="21" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="37" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C37" s="82" t="s">
+      <c r="C37" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="62">
+      <c r="D37" s="50">
         <v>35000000000</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="21" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="38" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C38" s="82" t="s">
+      <c r="C38" s="70" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="81">
+      <c r="D38" s="69">
         <v>1</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="39" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C39" s="83" t="s">
+      <c r="C39" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="D39" s="85" t="s">
+      <c r="D39" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="E39" s="28"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="40" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C40" s="84"/>
-      <c r="D40" s="62"/>
-      <c r="E40" s="24"/>
+      <c r="C40" s="72"/>
+      <c r="D40" s="50"/>
     </row>
     <row r="41" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C41" s="87" t="s">
+      <c r="C41" s="75" t="s">
         <v>46</v>
       </c>
-      <c r="D41" s="88">
+      <c r="D41" s="76">
         <v>3500</v>
       </c>
-      <c r="E41" s="24"/>
     </row>
     <row r="42" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C42" s="84"/>
-      <c r="D42" s="81"/>
-      <c r="E42" s="24"/>
+      <c r="C42" s="72"/>
+      <c r="D42" s="69"/>
     </row>
     <row r="43" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C43" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D43" s="77" t="s">
+      <c r="D43" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="E43" s="50" t="s">
+      <c r="E43" s="42" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="44" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C44" s="45">
+      <c r="C44" s="3">
         <v>3</v>
       </c>
-      <c r="D44" s="62">
+      <c r="D44" s="50">
         <f>+$D$37*$D$36</f>
         <v>301667333.26386303</v>
       </c>
-      <c r="E44" s="86">
+      <c r="E44" s="74">
         <f>+D44*E24</f>
         <v>299793623.11936694</v>
       </c>
     </row>
     <row r="45" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C45" s="45">
+      <c r="C45" s="3">
         <f>+C44+3</f>
         <v>6</v>
       </c>
-      <c r="D45" s="62">
+      <c r="D45" s="50">
         <f t="shared" ref="D45:D46" si="5">+$D$37*$D$36</f>
         <v>301667333.26386303</v>
       </c>
-      <c r="E45" s="86">
+      <c r="E45" s="74">
         <f>+D45*E25</f>
         <v>297502301.04917461</v>
       </c>
     </row>
     <row r="46" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C46" s="45">
+      <c r="C46" s="3">
         <f>+C45+3</f>
         <v>9</v>
       </c>
-      <c r="D46" s="62">
+      <c r="D46" s="50">
         <f t="shared" si="5"/>
         <v>301667333.26386303</v>
       </c>
-      <c r="E46" s="86">
+      <c r="E46" s="74">
         <f>+D46*E26</f>
         <v>294812932.58134669</v>
       </c>
     </row>
     <row r="47" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C47" s="45">
+      <c r="C47" s="3">
         <f t="shared" ref="C47" si="6">+C46+3</f>
         <v>12</v>
       </c>
-      <c r="D47" s="62">
+      <c r="D47" s="50">
         <f>+$D$37*$D$36+D37</f>
         <v>35301667333.263863</v>
       </c>
-      <c r="E47" s="86">
+      <c r="E47" s="74">
         <f>+D47*E27</f>
         <v>34107891143.250111</v>
       </c>
     </row>
     <row r="48" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C48" s="26"/>
-      <c r="D48" s="78" t="s">
+      <c r="C48" s="23"/>
+      <c r="D48" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="E48" s="56">
+      <c r="E48" s="46">
         <f>SUM(E44:E47)</f>
         <v>35000000000</v>
       </c>
@@ -8954,10 +8867,10 @@
       <c r="C50" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D50" s="77" t="s">
+      <c r="D50" s="65" t="s">
         <v>42</v>
       </c>
-      <c r="E50" s="50" t="s">
+      <c r="E50" s="42" t="s">
         <v>78</v>
       </c>
       <c r="F50" s="2" t="s">
@@ -8966,164 +8879,146 @@
       <c r="G50" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H50" s="50" t="s">
+      <c r="H50" s="42" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="51" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C51" s="45">
+      <c r="C51" s="3">
         <v>3</v>
       </c>
-      <c r="D51" s="62">
+      <c r="D51" s="50">
         <f>+$D$35*(J24*0.25)</f>
         <v>8000</v>
       </c>
-      <c r="E51" s="86">
+      <c r="E51" s="74">
         <f>+D51*I24</f>
         <v>7993.6051159072749</v>
       </c>
-      <c r="F51" s="90">
+      <c r="F51" s="78">
         <f>+$D$41*(1+D24*C24/12)/(1+H24*G24/12)</f>
         <v>3519.0597521982422</v>
       </c>
-      <c r="G51" s="62">
+      <c r="G51" s="50">
         <f>+F51*D51</f>
         <v>28152478.017585937</v>
       </c>
-      <c r="H51" s="86">
+      <c r="H51" s="74">
         <f>+G51*E24</f>
         <v>27977617.905675463</v>
       </c>
     </row>
     <row r="52" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C52" s="45">
+      <c r="C52" s="3">
         <f>+C51+3</f>
         <v>6</v>
       </c>
-      <c r="D52" s="62">
+      <c r="D52" s="50">
         <f>+$D$35*(J25*0.25)</f>
         <v>9492.4060751400139</v>
       </c>
-      <c r="E52" s="86">
+      <c r="E52" s="74">
         <f>+D52*I25</f>
         <v>9475.8233842176342</v>
       </c>
-      <c r="F52" s="90">
+      <c r="F52" s="78">
         <f>+$D$41*(1+D25*C25/12)/(1+H25*G25/12)</f>
         <v>3542.800099825306</v>
       </c>
-      <c r="G52" s="62">
+      <c r="G52" s="50">
         <f t="shared" ref="G52:G54" si="7">+F52*D52</f>
         <v>33629697.190588385</v>
       </c>
-      <c r="H52" s="86">
+      <c r="H52" s="74">
         <f>+G52*E25</f>
         <v>33165381.844761722</v>
       </c>
     </row>
     <row r="53" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C53" s="45">
+      <c r="C53" s="3">
         <f>+C52+3</f>
         <v>9</v>
       </c>
-      <c r="D53" s="62">
+      <c r="D53" s="50">
         <f>+$D$35*(J26*0.25)</f>
         <v>10980.783628651292</v>
       </c>
-      <c r="E53" s="86">
+      <c r="E53" s="74">
         <f>+D53*I26</f>
         <v>10949.577333251524</v>
       </c>
-      <c r="F53" s="90">
+      <c r="F53" s="78">
         <f>+$D$41*(1+D26*C26/12)/(1+H26*G26/12)</f>
         <v>3571.1970882983496</v>
       </c>
-      <c r="G53" s="62">
+      <c r="G53" s="50">
         <f t="shared" si="7"/>
         <v>39214542.521873683</v>
       </c>
-      <c r="H53" s="86">
+      <c r="H53" s="74">
         <f>+G53*E26</f>
         <v>38323520.666380338</v>
       </c>
     </row>
     <row r="54" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C54" s="45">
+      <c r="C54" s="3">
         <f t="shared" ref="C54" si="8">+C53+3</f>
         <v>12</v>
       </c>
-      <c r="D54" s="62">
+      <c r="D54" s="50">
         <f>+$D$35*(J27*0.25)+D35</f>
         <v>10011467.318143291</v>
       </c>
-      <c r="E54" s="86">
+      <c r="E54" s="74">
         <f>+D54*I27</f>
         <v>9971580.9941666257</v>
       </c>
-      <c r="F54" s="90">
+      <c r="F54" s="78">
         <f>+$D$41*(1+D27*C27/12)/(1+H27*G27/12)</f>
         <v>3608.0677290836647</v>
       </c>
-      <c r="G54" s="62">
+      <c r="G54" s="50">
         <f t="shared" si="7"/>
         <v>36122052151.368591</v>
       </c>
-      <c r="H54" s="86">
+      <c r="H54" s="74">
         <f>+G54*E27</f>
         <v>34900533479.583183</v>
       </c>
     </row>
     <row r="55" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C55" s="26"/>
-      <c r="D55" s="78" t="s">
+      <c r="C55" s="23"/>
+      <c r="D55" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="E55" s="56">
+      <c r="E55" s="46">
         <f>SUM(E51:E54)</f>
         <v>10000000.000000002</v>
       </c>
-      <c r="F55" s="91"/>
-      <c r="G55" s="78" t="s">
+      <c r="F55" s="79"/>
+      <c r="G55" s="66" t="s">
         <v>28</v>
       </c>
-      <c r="H55" s="107">
+      <c r="H55" s="95">
         <f>SUM(H51:H54)</f>
         <v>35000000000</v>
       </c>
     </row>
-    <row r="56" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="24"/>
-      <c r="F56" s="24"/>
-      <c r="G56" s="24"/>
-      <c r="H56" s="24"/>
-    </row>
     <row r="57" spans="3:8" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="C57" s="24"/>
-      <c r="D57" s="92" t="s">
+      <c r="D57" s="80" t="s">
         <v>93</v>
       </c>
-      <c r="E57" s="88">
+      <c r="E57" s="76">
         <f>+E55*D41-E48</f>
         <v>0</v>
       </c>
-      <c r="F57" s="24"/>
-      <c r="G57" s="92" t="s">
+      <c r="G57" s="80" t="s">
         <v>93</v>
       </c>
-      <c r="H57" s="88">
+      <c r="H57" s="76">
         <f>+H55-E48</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="C58" s="24"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="24"/>
-      <c r="G58" s="24"/>
-      <c r="H58" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>